<commit_message>
content: import latest Goodreads export
- Glorious Exploits: currently-reading -> read (3 stars)
- New reads: Whistler (Ann Patchett), Demian (Hermann Hesse)
- Now reading: The King Must Die (Mary Renault)
- Regenerate shelf.json and currently-reading.json

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCAL9FzbansxseAwbZAk9M
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD729"/>
+  <dimension ref="A1:AD732"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -67099,7 +67099,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1776505070i/69819.jpg</v>
       </c>
       <c r="AD725" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="726">
@@ -67283,7 +67283,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1604069900i/55077697.jpg</v>
       </c>
       <c r="AD727" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="728">
@@ -67375,7 +67375,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1754068063i/231387262.jpg</v>
       </c>
       <c r="AD728" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="729">
@@ -67401,7 +67401,7 @@
         <v>9781250893697</v>
       </c>
       <c r="H729">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I729" t="str">
         <v>Henry Holt and Co.</v>
@@ -67418,8 +67418,8 @@
       <c r="M729">
         <v>2024</v>
       </c>
-      <c r="N729" t="str">
-        <v/>
+      <c r="N729" s="1" t="d">
+        <v>2026-08-31T00:00:00.000Z</v>
       </c>
       <c r="O729" s="1" t="d">
         <v>2024-11-14T00:00:00.000Z</v>
@@ -67431,7 +67431,7 @@
         <v>currently-reading (#1), 2026 (#34)</v>
       </c>
       <c r="R729" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S729" t="str">
         <v/>
@@ -67470,9 +67470,285 @@
         <v>Mine</v>
       </c>
     </row>
+    <row r="730">
+      <c r="A730">
+        <v>242693052</v>
+      </c>
+      <c r="B730" t="str">
+        <v>Whistler</v>
+      </c>
+      <c r="C730" t="str">
+        <v>Ann Patchett</v>
+      </c>
+      <c r="D730" t="str">
+        <v>Patchett, Ann</v>
+      </c>
+      <c r="E730" t="str">
+        <v/>
+      </c>
+      <c r="F730" t="str">
+        <v>0063511630</v>
+      </c>
+      <c r="G730" t="str">
+        <v>9780063511637</v>
+      </c>
+      <c r="H730">
+        <v>3</v>
+      </c>
+      <c r="I730" t="str">
+        <v>Harper</v>
+      </c>
+      <c r="J730" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K730">
+        <v>304</v>
+      </c>
+      <c r="L730">
+        <v>2026</v>
+      </c>
+      <c r="M730">
+        <v>2026</v>
+      </c>
+      <c r="N730" s="1" t="d">
+        <v>2026-09-06T00:00:00.000Z</v>
+      </c>
+      <c r="O730" s="1" t="d">
+        <v>2026-06-05T00:00:00.000Z</v>
+      </c>
+      <c r="P730">
+        <v>2026</v>
+      </c>
+      <c r="Q730" t="str">
+        <v>2026 (#36)</v>
+      </c>
+      <c r="R730" t="str">
+        <v>read</v>
+      </c>
+      <c r="S730" t="str">
+        <v/>
+      </c>
+      <c r="T730" t="str">
+        <v/>
+      </c>
+      <c r="U730" t="str">
+        <v/>
+      </c>
+      <c r="V730">
+        <v>1</v>
+      </c>
+      <c r="W730">
+        <v>0</v>
+      </c>
+      <c r="X730" t="str">
+        <v>Female</v>
+      </c>
+      <c r="Y730" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z730" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA730" t="str">
+        <v>USA</v>
+      </c>
+      <c r="AB730" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC730" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1761863582i/242693052.jpg</v>
+      </c>
+      <c r="AD730" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731">
+        <v>1573373</v>
+      </c>
+      <c r="B731" t="str">
+        <v>Demian: The Story of Emil Sinclair's Youth</v>
+      </c>
+      <c r="C731" t="str">
+        <v>Hermann Hesse</v>
+      </c>
+      <c r="D731" t="str">
+        <v>Hesse, Hermann</v>
+      </c>
+      <c r="E731" t="str">
+        <v>Michael Roloff, Michael Lebeck</v>
+      </c>
+      <c r="F731" t="str">
+        <v>0553262467</v>
+      </c>
+      <c r="G731" t="str">
+        <v>9780553262469</v>
+      </c>
+      <c r="H731">
+        <v>4</v>
+      </c>
+      <c r="I731" t="str">
+        <v xml:space="preserve">Bantam Books </v>
+      </c>
+      <c r="J731" t="str">
+        <v>Mass Market Paperback</v>
+      </c>
+      <c r="K731">
+        <v>142</v>
+      </c>
+      <c r="L731">
+        <v>1981</v>
+      </c>
+      <c r="M731">
+        <v>1919</v>
+      </c>
+      <c r="N731" s="1" t="d">
+        <v>2026-09-03T00:00:00.000Z</v>
+      </c>
+      <c r="O731" s="1" t="d">
+        <v>2026-09-01T00:00:00.000Z</v>
+      </c>
+      <c r="P731">
+        <v>2026</v>
+      </c>
+      <c r="Q731" t="str">
+        <v>2026 (#35)</v>
+      </c>
+      <c r="R731" t="str">
+        <v>read</v>
+      </c>
+      <c r="S731" t="str">
+        <v/>
+      </c>
+      <c r="T731" t="str">
+        <v/>
+      </c>
+      <c r="U731" t="str">
+        <v/>
+      </c>
+      <c r="V731">
+        <v>1</v>
+      </c>
+      <c r="W731">
+        <v>0</v>
+      </c>
+      <c r="X731" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y731" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z731" t="str">
+        <v>Bildungsroman</v>
+      </c>
+      <c r="AA731" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="AB731" t="str">
+        <v>German</v>
+      </c>
+      <c r="AC731" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1669191812i/1573373.jpg</v>
+      </c>
+      <c r="AD731" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732">
+        <v>1932696</v>
+      </c>
+      <c r="B732" t="str">
+        <v>The King Must Die</v>
+      </c>
+      <c r="C732" t="str">
+        <v>Mary Renault</v>
+      </c>
+      <c r="D732" t="str">
+        <v>Renault, Mary</v>
+      </c>
+      <c r="E732" t="str">
+        <v/>
+      </c>
+      <c r="F732" t="str">
+        <v/>
+      </c>
+      <c r="G732" t="str">
+        <v/>
+      </c>
+      <c r="H732">
+        <v>0</v>
+      </c>
+      <c r="I732" t="str">
+        <v>Pantheon (NYC)</v>
+      </c>
+      <c r="J732" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K732">
+        <v>338</v>
+      </c>
+      <c r="L732">
+        <v>1958</v>
+      </c>
+      <c r="M732">
+        <v>1958</v>
+      </c>
+      <c r="N732" t="str">
+        <v/>
+      </c>
+      <c r="O732" s="1" t="d">
+        <v>2020-11-15T00:00:00.000Z</v>
+      </c>
+      <c r="P732" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q732" t="str">
+        <v>currently-reading (#1), 2026 (#37)</v>
+      </c>
+      <c r="R732" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S732" t="str">
+        <v/>
+      </c>
+      <c r="T732" t="str">
+        <v/>
+      </c>
+      <c r="U732" t="str">
+        <v/>
+      </c>
+      <c r="V732">
+        <v>1</v>
+      </c>
+      <c r="W732">
+        <v>0</v>
+      </c>
+      <c r="X732" t="str">
+        <v>Female</v>
+      </c>
+      <c r="Y732" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z732" t="str">
+        <v>Historical Fiction</v>
+      </c>
+      <c r="AA732" t="str">
+        <v>UK</v>
+      </c>
+      <c r="AB732" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC732" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1347202341i/1932696.jpg</v>
+      </c>
+      <c r="AD732" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD729"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD732"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
content: import Goodreads export, add draft stubs for King Must Die and By Night in Chile
Also fix importer CSV decoding (codepage 65001).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD732"/>
+  <dimension ref="A1:AD734"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -67467,7 +67467,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1691418622i/127278133.jpg</v>
       </c>
       <c r="AD729" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="730">
@@ -67559,7 +67559,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1761863582i/242693052.jpg</v>
       </c>
       <c r="AD730" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="731">
@@ -67651,7 +67651,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1669191812i/1573373.jpg</v>
       </c>
       <c r="AD731" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="732">
@@ -67677,7 +67677,7 @@
         <v/>
       </c>
       <c r="H732">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I732" t="str">
         <v>Pantheon (NYC)</v>
@@ -67694,8 +67694,8 @@
       <c r="M732">
         <v>1958</v>
       </c>
-      <c r="N732" t="str">
-        <v/>
+      <c r="N732" s="1" t="d">
+        <v>2026-09-15T00:00:00.000Z</v>
       </c>
       <c r="O732" s="1" t="d">
         <v>2020-11-15T00:00:00.000Z</v>
@@ -67707,7 +67707,7 @@
         <v>currently-reading (#1), 2026 (#37)</v>
       </c>
       <c r="R732" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S732" t="str">
         <v/>
@@ -67746,9 +67746,193 @@
         <v>Mine</v>
       </c>
     </row>
+    <row r="733">
+      <c r="A733">
+        <v>15719405</v>
+      </c>
+      <c r="B733" t="str">
+        <v>By Night in Chile</v>
+      </c>
+      <c r="C733" t="str">
+        <v>Roberto Bolaño</v>
+      </c>
+      <c r="D733" t="str">
+        <v>Bolaño, Roberto</v>
+      </c>
+      <c r="E733" t="str">
+        <v>Chris    Andrews</v>
+      </c>
+      <c r="F733" t="str">
+        <v/>
+      </c>
+      <c r="G733" t="str">
+        <v/>
+      </c>
+      <c r="H733">
+        <v>2</v>
+      </c>
+      <c r="I733" t="str">
+        <v xml:space="preserve">New Directions </v>
+      </c>
+      <c r="J733" t="str">
+        <v>Paperback</v>
+      </c>
+      <c r="K733">
+        <v>130</v>
+      </c>
+      <c r="L733">
+        <v>2003</v>
+      </c>
+      <c r="M733">
+        <v>2000</v>
+      </c>
+      <c r="N733" s="1" t="d">
+        <v>2026-09-19T00:00:00.000Z</v>
+      </c>
+      <c r="O733" s="1" t="d">
+        <v>2026-09-19T00:00:00.000Z</v>
+      </c>
+      <c r="P733">
+        <v>2026</v>
+      </c>
+      <c r="Q733" t="str">
+        <v>2026 (#39)</v>
+      </c>
+      <c r="R733" t="str">
+        <v>read</v>
+      </c>
+      <c r="S733" t="str">
+        <v/>
+      </c>
+      <c r="T733" t="str">
+        <v/>
+      </c>
+      <c r="U733" t="str">
+        <v/>
+      </c>
+      <c r="V733">
+        <v>1</v>
+      </c>
+      <c r="W733">
+        <v>0</v>
+      </c>
+      <c r="X733" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y733" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z733" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA733" t="str">
+        <v>Chile</v>
+      </c>
+      <c r="AB733" t="str">
+        <v>Spanish</v>
+      </c>
+      <c r="AC733" t="str">
+        <v>https://covers.openlibrary.org/b/id/5381371-L.jpg</v>
+      </c>
+      <c r="AD733" t="str">
+        <v>Claude</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734">
+        <v>231127410</v>
+      </c>
+      <c r="B734" t="str">
+        <v>Alexander: God, King, Man</v>
+      </c>
+      <c r="C734" t="str">
+        <v>Edmund  Richardson</v>
+      </c>
+      <c r="D734" t="str">
+        <v>Richardson, Edmund</v>
+      </c>
+      <c r="E734" t="str">
+        <v/>
+      </c>
+      <c r="F734" t="str">
+        <v>1250285615</v>
+      </c>
+      <c r="G734" t="str">
+        <v>9781250285614</v>
+      </c>
+      <c r="H734">
+        <v>0</v>
+      </c>
+      <c r="I734" t="str">
+        <v>St. Martin's Press</v>
+      </c>
+      <c r="J734" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K734">
+        <v>480</v>
+      </c>
+      <c r="L734">
+        <v>2026</v>
+      </c>
+      <c r="M734">
+        <v>2026</v>
+      </c>
+      <c r="N734" t="str">
+        <v/>
+      </c>
+      <c r="O734" s="1" t="d">
+        <v>2026-08-21T00:00:00.000Z</v>
+      </c>
+      <c r="P734" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q734" t="str">
+        <v>currently-reading (#1), 2026 (#38)</v>
+      </c>
+      <c r="R734" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S734" t="str">
+        <v/>
+      </c>
+      <c r="T734" t="str">
+        <v/>
+      </c>
+      <c r="U734" t="str">
+        <v/>
+      </c>
+      <c r="V734">
+        <v>1</v>
+      </c>
+      <c r="W734">
+        <v>0</v>
+      </c>
+      <c r="X734" t="str">
+        <v/>
+      </c>
+      <c r="Y734" t="str">
+        <v/>
+      </c>
+      <c r="Z734" t="str">
+        <v/>
+      </c>
+      <c r="AA734" t="str">
+        <v/>
+      </c>
+      <c r="AB734" t="str">
+        <v/>
+      </c>
+      <c r="AC734" t="str">
+        <v/>
+      </c>
+      <c r="AD734" t="str">
+        <v>None</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD732"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD734"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
content: add covers for Chile and Alexander; publish Whistler review and Sept newsletter
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -67832,10 +67832,10 @@
         <v>Spanish</v>
       </c>
       <c r="AC733" t="str">
-        <v>https://covers.openlibrary.org/b/id/5381371-L.jpg</v>
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1340496323i/15719405.jpg</v>
       </c>
       <c r="AD733" t="str">
-        <v>Claude</v>
+        <v>Mine</v>
       </c>
     </row>
     <row r="734">
@@ -67924,10 +67924,10 @@
         <v/>
       </c>
       <c r="AC734" t="str">
-        <v/>
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1745184317i/231127410.jpg</v>
       </c>
       <c r="AD734" t="str">
-        <v>None</v>
+        <v>Mine</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content: import Goodreads export, finish Alexander, start American Hagwon
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD734"/>
+  <dimension ref="A1:AD735"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -67743,7 +67743,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1347202341i/1932696.jpg</v>
       </c>
       <c r="AD732" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="733">
@@ -67835,7 +67835,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1340496323i/15719405.jpg</v>
       </c>
       <c r="AD733" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="734">
@@ -67861,7 +67861,7 @@
         <v>9781250285614</v>
       </c>
       <c r="H734">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I734" t="str">
         <v>St. Martin's Press</v>
@@ -67878,8 +67878,8 @@
       <c r="M734">
         <v>2026</v>
       </c>
-      <c r="N734" t="str">
-        <v/>
+      <c r="N734" s="1" t="d">
+        <v>2026-09-30T00:00:00.000Z</v>
       </c>
       <c r="O734" s="1" t="d">
         <v>2026-08-21T00:00:00.000Z</v>
@@ -67891,7 +67891,7 @@
         <v>currently-reading (#1), 2026 (#38)</v>
       </c>
       <c r="R734" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S734" t="str">
         <v/>
@@ -67909,19 +67909,19 @@
         <v>0</v>
       </c>
       <c r="X734" t="str">
-        <v/>
+        <v>Male</v>
       </c>
       <c r="Y734" t="str">
-        <v/>
+        <v>Non-Fiction</v>
       </c>
       <c r="Z734" t="str">
-        <v/>
+        <v>Biography, History</v>
       </c>
       <c r="AA734" t="str">
-        <v/>
+        <v>United Kingdom</v>
       </c>
       <c r="AB734" t="str">
-        <v/>
+        <v>English</v>
       </c>
       <c r="AC734" t="str">
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1745184317i/231127410.jpg</v>
@@ -67930,9 +67930,101 @@
         <v>Mine</v>
       </c>
     </row>
+    <row r="735">
+      <c r="A735">
+        <v>245957901</v>
+      </c>
+      <c r="B735" t="str">
+        <v>American Hagwon</v>
+      </c>
+      <c r="C735" t="str">
+        <v>Min Jin Lee</v>
+      </c>
+      <c r="D735" t="str">
+        <v>Lee, Min Jin</v>
+      </c>
+      <c r="E735" t="str">
+        <v/>
+      </c>
+      <c r="F735" t="str">
+        <v>1538752042</v>
+      </c>
+      <c r="G735" t="str">
+        <v>9781538752043</v>
+      </c>
+      <c r="H735">
+        <v>0</v>
+      </c>
+      <c r="I735" t="str">
+        <v>Cardinal</v>
+      </c>
+      <c r="J735" t="str">
+        <v>ebook</v>
+      </c>
+      <c r="K735">
+        <v>656</v>
+      </c>
+      <c r="L735">
+        <v>2026</v>
+      </c>
+      <c r="M735">
+        <v>2026</v>
+      </c>
+      <c r="N735" t="str">
+        <v/>
+      </c>
+      <c r="O735" s="1" t="d">
+        <v>2026-08-21T00:00:00.000Z</v>
+      </c>
+      <c r="P735" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q735" t="str">
+        <v>currently-reading (#1), 2026 (#40)</v>
+      </c>
+      <c r="R735" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S735" t="str">
+        <v/>
+      </c>
+      <c r="T735" t="str">
+        <v/>
+      </c>
+      <c r="U735" t="str">
+        <v/>
+      </c>
+      <c r="V735">
+        <v>1</v>
+      </c>
+      <c r="W735">
+        <v>0</v>
+      </c>
+      <c r="X735" t="str">
+        <v>Female</v>
+      </c>
+      <c r="Y735" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z735" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA735" t="str">
+        <v>South Korea</v>
+      </c>
+      <c r="AB735" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC735" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1771958472i/245886309.jpg</v>
+      </c>
+      <c r="AD735" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD734"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD735"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>